<commit_message>
fix fip_ZQ9_VALMETH fixture headers to match real ZQ9_VALMETH export
Co-Authored-By: Claude Sonnet 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/test_data/fixtures/fip_ZQ9_VALMETH.xlsx
+++ b/test_data/fixtures/fip_ZQ9_VALMETH.xlsx
@@ -429,17 +429,17 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>Medium Text MK</t>
+          <t>Medium Text</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>Normal X-Check No</t>
+          <t>ValidRule</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>X-Check Medium Text</t>
+          <t>Medium Text</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
@@ -449,12 +449,12 @@
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>Condition No</t>
+          <t>ValidRule</t>
         </is>
       </c>
       <c r="H1" t="inlineStr">
         <is>
-          <t>Condition Medium Text</t>
+          <t>Medium Text</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
v1.0.36: add differences-mode fixtures and test cases (X-Check selection + Conditions yellow cell)
Co-Authored-By: Claude Sonnet 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/test_data/fixtures/fip_ZQ9_VALMETH.xlsx
+++ b/test_data/fixtures/fip_ZQ9_VALMETH.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H3"/>
+  <dimension ref="A1:H4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -537,6 +537,48 @@
         </is>
       </c>
       <c r="H3" t="inlineStr">
+        <is>
+          <t>Quarter 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>MK1</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Test MK</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>COND_DIFF_YELLOW</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Diff yellow test</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Q1</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
         <is>
           <t>Quarter 1</t>
         </is>

</xml_diff>

<commit_message>
v1.0.37: add green-cell Conditions fixture; fix green rule to check condition cell not col-A
Co-Authored-By: Claude Sonnet 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/test_data/fixtures/fip_ZQ9_VALMETH.xlsx
+++ b/test_data/fixtures/fip_ZQ9_VALMETH.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H4"/>
+  <dimension ref="A1:H5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -579,6 +579,48 @@
         </is>
       </c>
       <c r="H4" t="inlineStr">
+        <is>
+          <t>Quarter 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>MK1</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Test MK</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>COND_DIFF_GREEN</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Diff green test</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Q1</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
         <is>
           <t>Quarter 1</t>
         </is>

</xml_diff>